<commit_message>
Obsidian Vault Backup - 18-09-2026 10:02:27.59
</commit_message>
<xml_diff>
--- a/ISMS/PGDM FY ( TREAM 1)/Excel training/CLG SOURCE/practical pratice.xlsx
+++ b/ISMS/PGDM FY ( TREAM 1)/Excel training/CLG SOURCE/practical pratice.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\OneDrive\Documents\Obsidian Vault\ISMS\PGDM FY ( TREAM 1)\Excel training\CLG SOURCE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FD7DC09-6C27-4972-8D5C-6F3D0ABF1C93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{778929FA-F5E3-4F45-831B-234F087C8059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" activeTab="2" xr2:uid="{E8899D08-E41A-4E73-A0BC-0A1E6DFFE7E2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" activeTab="3" xr2:uid="{E8899D08-E41A-4E73-A0BC-0A1E6DFFE7E2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="83">
   <si>
     <t>Regine</t>
   </si>
@@ -209,6 +210,84 @@
   </si>
   <si>
     <t>Kushal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name </t>
+  </si>
+  <si>
+    <t>Dept</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sr no. </t>
+  </si>
+  <si>
+    <t>Ajay</t>
+  </si>
+  <si>
+    <t>Vijay</t>
+  </si>
+  <si>
+    <t>Praful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mehul </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rekha </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Esat </t>
+  </si>
+  <si>
+    <t>West</t>
+  </si>
+  <si>
+    <t>South</t>
+  </si>
+  <si>
+    <t>East</t>
+  </si>
+  <si>
+    <t>North</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grade </t>
+  </si>
+  <si>
+    <t>EXCELLENT</t>
+  </si>
+  <si>
+    <t>POOR</t>
+  </si>
+  <si>
+    <t>Expencec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regin </t>
+  </si>
+  <si>
+    <t>points</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>Leves</t>
+  </si>
+  <si>
+    <t>Rahul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ram </t>
+  </si>
+  <si>
+    <t>Raj</t>
+  </si>
+  <si>
+    <t>Rekha</t>
+  </si>
+  <si>
+    <t>Vijaya</t>
   </si>
 </sst>
 </file>
@@ -258,7 +337,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -268,6 +347,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -395,15 +480,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="justify"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -458,125 +540,147 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="40">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+  <dxfs count="53">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
         <right style="thin">
           <color indexed="64"/>
         </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
         <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -674,7 +778,139 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -695,6 +931,235 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -743,7 +1208,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -759,7 +1224,30 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -769,7 +1257,9 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom/>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -790,79 +1280,12 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -890,31 +1313,43 @@
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
+        <top/>
         <bottom/>
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -922,30 +1357,99 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom/>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
@@ -957,321 +1461,6 @@
         <top/>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1287,18 +1476,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61AC78F9-9CBB-43D5-ADEC-73925900EAE3}" name="Table1" displayName="Table1" ref="A1:G9" totalsRowShown="0" headerRowDxfId="33" dataDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61AC78F9-9CBB-43D5-ADEC-73925900EAE3}" name="Table1" displayName="Table1" ref="A1:G9" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
   <autoFilter ref="A1:G9" xr:uid="{61AC78F9-9CBB-43D5-ADEC-73925900EAE3}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{6DFA14BB-6073-48AA-892D-1FC5FAC205D3}" name="sr no." dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{09B0D5CB-3854-4C9A-A755-5B9E177267C3}" name="Name" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{9ED161A3-37DD-49E4-A9F1-E32B2A4B49D3}" name=" direction's " dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{AE6C2120-A53D-479B-8D85-B4515A2F7EC0}" name="Sales" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{CA10C443-6CA9-442E-9D43-BB794F3CDEBC}" name="CC" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{E1229AD3-A6F3-4425-A941-D6720C900C43}" name="Bones" dataDxfId="19">
+    <tableColumn id="1" xr3:uid="{6DFA14BB-6073-48AA-892D-1FC5FAC205D3}" name="sr no." dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{09B0D5CB-3854-4C9A-A755-5B9E177267C3}" name="Name" dataDxfId="41"/>
+    <tableColumn id="3" xr3:uid="{9ED161A3-37DD-49E4-A9F1-E32B2A4B49D3}" name=" direction's " dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{AE6C2120-A53D-479B-8D85-B4515A2F7EC0}" name="Sales" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{CA10C443-6CA9-442E-9D43-BB794F3CDEBC}" name="CC" dataDxfId="38"/>
+    <tableColumn id="6" xr3:uid="{E1229AD3-A6F3-4425-A941-D6720C900C43}" name="Bones" dataDxfId="37">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[Sales]]&lt;=$I$14,Table1[[#This Row],[CC]]&lt;=$I$15),$I$16,$I$17)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{4B7AF343-BC89-469D-920A-3FE880B5BC86}" name="change in polices" dataDxfId="32">
+    <tableColumn id="7" xr3:uid="{4B7AF343-BC89-469D-920A-3FE880B5BC86}" name="change in polices" dataDxfId="36">
       <calculatedColumnFormula>IF(AND(Table1[[#This Row],[Sales]]&gt;=$I$14,Table1[[#This Row],[CC]]&lt;=$I$15),$I$16,$I$17)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1307,20 +1496,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{88CD5FDC-F6E4-4348-B2D1-DDB18D1EFD35}" name="Table3" displayName="Table3" ref="A21:I30" totalsRowCount="1" headerRowDxfId="20" dataDxfId="21" headerRowBorderDxfId="30" tableBorderDxfId="31" totalsRowBorderDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{88CD5FDC-F6E4-4348-B2D1-DDB18D1EFD35}" name="Table3" displayName="Table3" ref="A21:I30" totalsRowCount="1" headerRowDxfId="35" dataDxfId="33" headerRowBorderDxfId="34" tableBorderDxfId="32" totalsRowBorderDxfId="31">
   <autoFilter ref="A21:I29" xr:uid="{88CD5FDC-F6E4-4348-B2D1-DDB18D1EFD35}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{D051F378-3107-4931-A5C2-418D1C1AE30B}" name="sr no." totalsRowLabel="Total" dataDxfId="28" totalsRowDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{7BAA1871-2C8B-4AC4-9301-02674506F2EA}" name="Name" dataDxfId="27" totalsRowDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{4B282B04-5C37-4CB1-ACBC-E766F2B6AD94}" name=" direction's " dataDxfId="26" totalsRowDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{71A96920-2B0A-4695-BADD-15FCB6767D55}" name="Sales" dataDxfId="25" totalsRowDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{32D1D996-5584-4B91-8837-437B25581DA0}" name="CC" dataDxfId="24" totalsRowDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{990DBAAE-213E-46FF-AB83-35CF8367987D}" name="Bones" totalsRowFunction="custom" dataDxfId="23" totalsRowDxfId="17">
+    <tableColumn id="1" xr3:uid="{D051F378-3107-4931-A5C2-418D1C1AE30B}" name="sr no." totalsRowLabel="Total" dataDxfId="30" totalsRowDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{7BAA1871-2C8B-4AC4-9301-02674506F2EA}" name="Name" dataDxfId="28" totalsRowDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{4B282B04-5C37-4CB1-ACBC-E766F2B6AD94}" name=" direction's " dataDxfId="26" totalsRowDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{71A96920-2B0A-4695-BADD-15FCB6767D55}" name="Sales" dataDxfId="24" totalsRowDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{32D1D996-5584-4B91-8837-437B25581DA0}" name="CC" dataDxfId="22" totalsRowDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{990DBAAE-213E-46FF-AB83-35CF8367987D}" name="Bones" totalsRowFunction="custom" dataDxfId="20" totalsRowDxfId="19">
       <totalsRowFormula>SUM(Table3[Bones])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{6F9363FD-06CA-42CE-830C-D878CCDCF0A8}" name="change in polices" totalsRowFunction="sum" dataDxfId="22" totalsRowDxfId="18"/>
-    <tableColumn id="8" xr3:uid="{9AC6E63C-8C4B-410A-9246-3E9FA8FA3E50}" name="expense" dataDxfId="11" totalsRowDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{746B59DF-7C34-475A-B6C6-E701F25F606E}" name="salary" dataDxfId="8" totalsRowDxfId="9">
+    <tableColumn id="7" xr3:uid="{6F9363FD-06CA-42CE-830C-D878CCDCF0A8}" name="change in polices" totalsRowFunction="sum" dataDxfId="18" totalsRowDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{9AC6E63C-8C4B-410A-9246-3E9FA8FA3E50}" name="expense" dataDxfId="16" totalsRowDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{746B59DF-7C34-475A-B6C6-E701F25F606E}" name="salary" dataDxfId="14" totalsRowDxfId="13">
       <calculatedColumnFormula>IF(AND(Table3[[#This Row],[expense]]&lt;$M$26,Table3[[#This Row],[expense]]&gt;$M$27),$M$28,$M$29)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1329,13 +1518,13 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D4534C78-F1C6-4118-92DF-B06685442D1B}" name="Table5" displayName="Table5" ref="A7:D11" totalsRowShown="0" headerRowDxfId="4" headerRowBorderDxfId="2" tableBorderDxfId="3" totalsRowBorderDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D4534C78-F1C6-4118-92DF-B06685442D1B}" name="Table5" displayName="Table5" ref="A7:D11" totalsRowShown="0" headerRowDxfId="52" headerRowBorderDxfId="51" tableBorderDxfId="50" totalsRowBorderDxfId="49">
   <autoFilter ref="A7:D11" xr:uid="{D4534C78-F1C6-4118-92DF-B06685442D1B}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{C3D5E930-74E8-492A-B72A-C8ED95AF5FC3}" name="First Name " dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{47254F64-0D29-4E9F-9720-783CAF5E222E}" name="midel name " dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{66406B99-7F8C-471C-B23D-6C7A761644A6}" name="last name" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{65B5B06B-98B5-4597-9BE4-1C75F2F85794}" name="full name " dataDxfId="0">
+    <tableColumn id="1" xr3:uid="{C3D5E930-74E8-492A-B72A-C8ED95AF5FC3}" name="First Name " dataDxfId="48"/>
+    <tableColumn id="2" xr3:uid="{47254F64-0D29-4E9F-9720-783CAF5E222E}" name="midel name " dataDxfId="47"/>
+    <tableColumn id="3" xr3:uid="{66406B99-7F8C-471C-B23D-6C7A761644A6}" name="last name" dataDxfId="46"/>
+    <tableColumn id="4" xr3:uid="{65B5B06B-98B5-4597-9BE4-1C75F2F85794}" name="full name " dataDxfId="45">
       <calculatedColumnFormula>_xlfn.CONCAT(Table5[[#This Row],[First Name ]],IF(Table5[[#This Row],[midel name ]]="",""," "),Table5[[#This Row],[midel name ]]," ",Table5[[#This Row],[last name]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2016,7 +2205,7 @@
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-      <c r="F10" s="3"/>
+      <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
@@ -2024,7 +2213,7 @@
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
-      <c r="F11" s="3"/>
+      <c r="F11" s="2"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="H14" t="s">
@@ -2058,181 +2247,181 @@
         <v>400</v>
       </c>
     </row>
-    <row r="21" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
+    <row r="21" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E21" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F21" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="G21" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="H21" s="10" t="s">
+      <c r="H21" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="I21" s="10" t="s">
+      <c r="I21" s="9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" s="7">
+      <c r="A22" s="6">
         <v>1</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="5">
         <v>5</v>
       </c>
-      <c r="E22" s="6">
+      <c r="E22" s="5">
         <v>8</v>
       </c>
-      <c r="F22" s="5">
+      <c r="F22" s="4">
         <v>400</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="7">
         <v>400</v>
       </c>
-      <c r="H22" s="16">
+      <c r="H22" s="15">
         <v>5</v>
       </c>
-      <c r="I22" s="16">
+      <c r="I22" s="15">
         <f>IF(AND(Table3[[#This Row],[expense]]&lt;$M$26,Table3[[#This Row],[expense]]&gt;$M$27),$M$28,$M$29)</f>
         <v>1000</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A23" s="7">
+      <c r="A23" s="6">
         <v>2</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="5">
         <v>9</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="5">
         <v>2</v>
       </c>
-      <c r="F23" s="5">
+      <c r="F23" s="4">
         <v>2000</v>
       </c>
-      <c r="G23" s="8">
+      <c r="G23" s="7">
         <v>2000</v>
       </c>
-      <c r="H23" s="6">
+      <c r="H23" s="5">
         <v>9</v>
       </c>
-      <c r="I23" s="6">
+      <c r="I23" s="5">
         <f>IF(AND(Table3[[#This Row],[expense]]&lt;$M$26,Table3[[#This Row],[expense]]&gt;$M$27),$M$28,$M$29)</f>
         <v>200</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A24" s="7">
+      <c r="A24" s="6">
         <v>3</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="5">
         <v>3</v>
       </c>
-      <c r="E24" s="6">
+      <c r="E24" s="5">
         <v>4</v>
       </c>
-      <c r="F24" s="5">
+      <c r="F24" s="4">
         <v>2000</v>
       </c>
-      <c r="G24" s="8">
+      <c r="G24" s="7">
         <v>400</v>
       </c>
-      <c r="H24" s="6">
+      <c r="H24" s="5">
         <v>3</v>
       </c>
-      <c r="I24" s="6">
+      <c r="I24" s="5">
         <f>IF(AND(Table3[[#This Row],[expense]]&lt;$M$26,Table3[[#This Row],[expense]]&gt;$M$27),$M$28,$M$29)</f>
         <v>200</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A25" s="7">
+      <c r="A25" s="6">
         <v>4</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="5">
         <v>4</v>
       </c>
-      <c r="E25" s="6">
+      <c r="E25" s="5">
         <v>7</v>
       </c>
-      <c r="F25" s="5">
+      <c r="F25" s="4">
         <v>2000</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="7">
         <v>400</v>
       </c>
-      <c r="H25" s="6">
+      <c r="H25" s="5">
         <v>4</v>
       </c>
-      <c r="I25" s="6">
+      <c r="I25" s="5">
         <f>IF(AND(Table3[[#This Row],[expense]]&lt;$M$26,Table3[[#This Row],[expense]]&gt;$M$27),$M$28,$M$29)</f>
         <v>200</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" s="7">
+      <c r="A26" s="6">
         <v>5</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="5">
         <v>7</v>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="5">
         <v>1</v>
       </c>
-      <c r="F26" s="5">
+      <c r="F26" s="4">
         <v>2000</v>
       </c>
-      <c r="G26" s="8">
+      <c r="G26" s="7">
         <v>2000</v>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="5">
         <v>7</v>
       </c>
-      <c r="I26" s="6">
+      <c r="I26" s="5">
         <f>IF(AND(Table3[[#This Row],[expense]]&lt;$M$26,Table3[[#This Row],[expense]]&gt;$M$27),$M$28,$M$29)</f>
         <v>200</v>
       </c>
@@ -2244,31 +2433,31 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A27" s="7">
+      <c r="A27" s="6">
         <v>6</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D27" s="6">
+      <c r="D27" s="5">
         <v>2</v>
       </c>
-      <c r="E27" s="6">
+      <c r="E27" s="5">
         <v>9</v>
       </c>
-      <c r="F27" s="5">
+      <c r="F27" s="4">
         <v>2000</v>
       </c>
-      <c r="G27" s="8">
+      <c r="G27" s="7">
         <v>400</v>
       </c>
-      <c r="H27" s="6">
+      <c r="H27" s="5">
         <v>2</v>
       </c>
-      <c r="I27" s="6">
+      <c r="I27" s="5">
         <f>IF(AND(Table3[[#This Row],[expense]]&lt;$M$26,Table3[[#This Row],[expense]]&gt;$M$27),$M$28,$M$29)</f>
         <v>200</v>
       </c>
@@ -2280,31 +2469,31 @@
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A28" s="7">
+      <c r="A28" s="6">
         <v>7</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D28" s="6">
+      <c r="D28" s="5">
         <v>1</v>
       </c>
-      <c r="E28" s="6">
+      <c r="E28" s="5">
         <v>2</v>
       </c>
-      <c r="F28" s="5">
+      <c r="F28" s="4">
         <v>2000</v>
       </c>
-      <c r="G28" s="8">
+      <c r="G28" s="7">
         <v>400</v>
       </c>
-      <c r="H28" s="6">
+      <c r="H28" s="5">
         <v>1</v>
       </c>
-      <c r="I28" s="6">
+      <c r="I28" s="5">
         <f>IF(AND(Table3[[#This Row],[expense]]&lt;$M$26,Table3[[#This Row],[expense]]&gt;$M$27),$M$28,$M$29)</f>
         <v>200</v>
       </c>
@@ -2316,31 +2505,31 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A29" s="12">
+      <c r="A29" s="11">
         <v>8</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="B29" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="D29" s="13">
+      <c r="D29" s="12">
         <v>4</v>
       </c>
-      <c r="E29" s="13">
+      <c r="E29" s="12">
         <v>6</v>
       </c>
-      <c r="F29" s="14">
+      <c r="F29" s="13">
         <v>2000</v>
       </c>
-      <c r="G29" s="15">
+      <c r="G29" s="14">
         <v>2000</v>
       </c>
-      <c r="H29" s="13">
+      <c r="H29" s="12">
         <v>4</v>
       </c>
-      <c r="I29" s="13">
+      <c r="I29" s="12">
         <f>IF(AND(Table3[[#This Row],[expense]]&lt;$M$26,Table3[[#This Row],[expense]]&gt;$M$27),$M$28,$M$29)</f>
         <v>200</v>
       </c>
@@ -2352,23 +2541,23 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="14">
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="13">
         <f>SUM(Table3[Bones])</f>
         <v>14400</v>
       </c>
-      <c r="G30" s="15">
+      <c r="G30" s="14">
         <f>SUBTOTAL(109,Table3[change in polices])</f>
         <v>8000</v>
       </c>
-      <c r="H30" s="13"/>
-      <c r="I30" s="13"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -2490,75 +2679,75 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="D8" s="19" t="str">
+      <c r="D8" s="18" t="str">
         <f>_xlfn.CONCAT(Table5[[#This Row],[First Name ]],IF(Table5[[#This Row],[midel name ]]="",""," "),Table5[[#This Row],[midel name ]]," ",Table5[[#This Row],[last name]])</f>
         <v>Rahul  Ram Kulkarni</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="19" t="str">
+      <c r="D9" s="18" t="str">
         <f>_xlfn.CONCAT(Table5[[#This Row],[First Name ]],IF(Table5[[#This Row],[midel name ]]="",""," "),Table5[[#This Row],[midel name ]]," ",Table5[[#This Row],[last name]])</f>
         <v>Uvi Kushal Sharma</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="19" t="str">
+      <c r="D10" s="18" t="str">
         <f>_xlfn.CONCAT(Table5[[#This Row],[First Name ]],IF(Table5[[#This Row],[midel name ]]="",""," "),Table5[[#This Row],[midel name ]]," ",Table5[[#This Row],[last name]])</f>
         <v>Kavya Ravi Mishra</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="19" t="str">
+      <c r="D11" s="18" t="str">
         <f>_xlfn.CONCAT(Table5[[#This Row],[First Name ]],IF(Table5[[#This Row],[midel name ]]="",""," "),Table5[[#This Row],[midel name ]]," ",Table5[[#This Row],[last name]])</f>
         <v>Dipak kumar  Thakur</v>
       </c>
@@ -2569,4 +2758,413 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{055D6EC0-B52E-4BE7-B8D9-CEBD5C8128C7}">
+  <dimension ref="A1:P42"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A1" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A2" s="23">
+        <v>1</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="23">
+        <v>4</v>
+      </c>
+      <c r="D2" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="E2" s="23">
+        <v>5</v>
+      </c>
+      <c r="F2" s="23" t="str">
+        <f>IF(E2&gt;$O$2,$P$2,$O$3)</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="O2">
+        <v>4</v>
+      </c>
+      <c r="P2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A3" s="23">
+        <v>2</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="23">
+        <v>3</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="E3" s="23">
+        <v>9</v>
+      </c>
+      <c r="F3" s="23" t="str">
+        <f>IF(E3&gt;$O$2,$P$2,$O$3)</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="O3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4" s="23">
+        <v>3</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="23">
+        <v>1</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" s="23">
+        <v>3</v>
+      </c>
+      <c r="F4" s="23" t="str">
+        <f>IF(E4&gt;$O$2,$P$2,$O$3)</f>
+        <v>POOR</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A5" s="23">
+        <v>4</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="23">
+        <v>4</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="23">
+        <v>4</v>
+      </c>
+      <c r="F5" s="23" t="str">
+        <f>IF(E5&gt;$O$2,$P$2,$O$3)</f>
+        <v>POOR</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A6" s="23">
+        <v>5</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="23">
+        <v>6</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" s="23">
+        <v>7</v>
+      </c>
+      <c r="F6" s="23" t="str">
+        <f>IF(E6&gt;$O$2,$P$2,$O$3)</f>
+        <v>EXCELLENT</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A7" s="23">
+        <v>6</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="23">
+        <v>4</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" s="23">
+        <v>2</v>
+      </c>
+      <c r="F7" s="23" t="str">
+        <f>IF(E7&gt;$O$2,$P$2,$O$3)</f>
+        <v>POOR</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A8" s="23">
+        <v>7</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="23">
+        <v>3</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="E8" s="23">
+        <v>1</v>
+      </c>
+      <c r="F8" s="23" t="str">
+        <f>IF(E8&gt;$O$2,$P$2,$O$3)</f>
+        <v>POOR</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A9" s="23">
+        <v>8</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="23">
+        <v>2</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="E9" s="23">
+        <v>4</v>
+      </c>
+      <c r="F9" s="23" t="str">
+        <f>IF(E9&gt;$O$2,$P$2,$O$3)</f>
+        <v>POOR</v>
+      </c>
+    </row>
+    <row r="18" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G18" t="s">
+        <v>74</v>
+      </c>
+      <c r="H18" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G19" t="s">
+        <v>68</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G20" t="s">
+        <v>66</v>
+      </c>
+      <c r="H20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G21" t="s">
+        <v>69</v>
+      </c>
+      <c r="H21">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G22" t="s">
+        <v>67</v>
+      </c>
+      <c r="H22">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="H23">
+        <f>SUM(H19:H22,MAX(H19:H22))</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35" s="23">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="23">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B37" s="23">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" s="23">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="B39" s="23">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="B40" s="23">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B41" s="23">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="B42" s="23">
+        <v>90</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E2:E9">
+    <cfRule type="dataBar" priority="7">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{57FF0803-FA33-4158-B3A8-F1084F91C10D}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C9">
+    <cfRule type="dataBar" priority="6">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{EF226BA4-27A9-4C6A-9BA0-965789B1A717}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A35:A42">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="notEqual">
+      <formula>"vijay"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+      <formula>"vijay"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
+      <formula>"Vijay"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B35:B42">
+    <cfRule type="uniqueValues" dxfId="0" priority="3"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{57FF0803-FA33-4158-B3A8-F1084F91C10D}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF63C384"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E2:E9</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{EF226BA4-27A9-4C6A-9BA0-965789B1A717}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>C2:C9</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>